<commit_message>
chore: fully remove pricing section
</commit_message>
<xml_diff>
--- a/data/contacts.xlsx
+++ b/data/contacts.xlsx
@@ -397,10 +397,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:F2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>email</v>
+      </c>
+      <c r="D1" t="str">
+        <v>phone</v>
+      </c>
+      <c r="E1" t="str">
+        <v>message</v>
+      </c>
+      <c r="F1" t="str">
+        <v>date</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>kydsle</v>
+      </c>
+      <c r="B2" t="str">
+        <v>andrew</v>
+      </c>
+      <c r="C2" t="str">
+        <v>bill@adnre.com</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2348920902</v>
+      </c>
+      <c r="E2" t="str">
+        <v>msg</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2026-06-11T15:46:21.032Z</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: full page mobile menu and dev script fix
</commit_message>
<xml_diff>
--- a/data/contacts.xlsx
+++ b/data/contacts.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -439,9 +439,89 @@
         <v>2026-06-11T15:46:21.032Z</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>onrswn</v>
+      </c>
+      <c r="B3" t="str">
+        <v>andrew</v>
+      </c>
+      <c r="C3" t="str">
+        <v>bill@yahoo.com</v>
+      </c>
+      <c r="D3" t="str">
+        <v>11912912011</v>
+      </c>
+      <c r="E3" t="str">
+        <v>hi</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-06-11T15:50:01.534Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>lxx65i</v>
+      </c>
+      <c r="B4" t="str">
+        <v>matt</v>
+      </c>
+      <c r="C4" t="str">
+        <v>matthenry@gmail.com</v>
+      </c>
+      <c r="D4" t="str">
+        <v>267328723</v>
+      </c>
+      <c r="E4" t="str">
+        <v>hi</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-06-11T15:50:55.015Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>p6jgzb</v>
+      </c>
+      <c r="B5" t="str">
+        <v>test</v>
+      </c>
+      <c r="C5" t="str">
+        <v>t@t.com</v>
+      </c>
+      <c r="D5" t="str">
+        <v>123</v>
+      </c>
+      <c r="E5" t="str">
+        <v>m</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-06-11T15:52:25.268Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>8tyges</v>
+      </c>
+      <c r="B6" t="str">
+        <v>matt</v>
+      </c>
+      <c r="C6" t="str">
+        <v>matthenry@gmail.com</v>
+      </c>
+      <c r="D6" t="str">
+        <v>267328723</v>
+      </c>
+      <c r="E6" t="str">
+        <v>hi</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2026-06-11T15:52:47.955Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: reset contact form and show beautiful success state for 3 seconds
</commit_message>
<xml_diff>
--- a/data/contacts.xlsx
+++ b/data/contacts.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -519,9 +519,49 @@
         <v>2026-06-11T15:52:47.955Z</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>824ed7</v>
+      </c>
+      <c r="B7" t="str">
+        <v>matt</v>
+      </c>
+      <c r="C7" t="str">
+        <v>matthenry@gmail.com</v>
+      </c>
+      <c r="D7" t="str">
+        <v>267328723</v>
+      </c>
+      <c r="E7" t="str">
+        <v>hi</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-06-11T15:54:13.007Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>4n92v8</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Mohan Prasath S</v>
+      </c>
+      <c r="C8" t="str">
+        <v>mohanprasath563@gmail.com</v>
+      </c>
+      <c r="D8" t="str">
+        <v>09025521149</v>
+      </c>
+      <c r="E8" t="str">
+        <v>hi</v>
+      </c>
+      <c r="F8" t="str">
+        <v>2026-06-11T15:54:45.625Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add 3 second simulated processing delay to contact forms
</commit_message>
<xml_diff>
--- a/data/contacts.xlsx
+++ b/data/contacts.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -559,9 +559,29 @@
         <v>2026-06-11T15:54:45.625Z</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>rhmrkh</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Mohan Prasath S</v>
+      </c>
+      <c r="C9" t="str">
+        <v>mohanprasath563@gmail.com</v>
+      </c>
+      <c r="D9" t="str">
+        <v>09025421149</v>
+      </c>
+      <c r="E9" t="str">
+        <v>hi</v>
+      </c>
+      <c r="F9" t="str">
+        <v>2026-06-11T15:57:42.220Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>